<commit_message>
feat: derive light output config from supported_color_modes via derive_fn hook
Replace the 4 dead light entries (device_class: None/brightness/color_temp/rgb)
with a single entry carrying a derive_fn callable. Add resolve_entity_mapping()
which merges derive_fn output at config time. Add 16 tests covering all tiers,
fallback cases, and the resolver.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ88"/>
+  <dimension ref="A1:AQ85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ha-light-onoff</t>
+          <t>ha-light</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -9121,22 +9121,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>lock</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>brightness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HA Light (brightness)</t>
+          <t>HA Lock</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ha-light-brightness</t>
+          <t>ha-lock-none</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -9151,7 +9151,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DOOR_OPEN</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ACCESS</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>DIMMER</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -9236,22 +9236,22 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>BINARY</t>
         </is>
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH47" t="inlineStr">
@@ -9308,22 +9308,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>number</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>color_temp</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HA Light (color_temp)</t>
+          <t>HA Number</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ha-light-color_temp</t>
+          <t>ha-number-none</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -9338,7 +9338,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>DIMMER_COLOR_TEMP</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB48" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -9438,12 +9438,12 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>POWER_LEVEL</t>
         </is>
       </c>
       <c r="AH48" t="inlineStr">
         <is>
-          <t>COLOR_TEMPERATURE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI48" t="inlineStr">
@@ -9495,22 +9495,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>rgb</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HA Light (rgb)</t>
+          <t>HA Sensor</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ha-light-rgb</t>
+          <t>ha-sensor-none</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -9560,32 +9560,50 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>100</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V49" t="n">
+        <v>30</v>
+      </c>
+      <c r="W49" t="n">
+        <v>120</v>
+      </c>
+      <c r="X49" t="n">
+        <v>2</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr">
@@ -9595,7 +9613,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>FULL_COLOR_DIMMER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -9605,52 +9623,52 @@
       </c>
       <c r="AC49" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>HUE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI49" t="inlineStr">
         <is>
-          <t>SATURATION</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>COLOR_TEMPERATURE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>CIE_X</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
-          <t>CIE_Y</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AM49" t="inlineStr">
@@ -9682,22 +9700,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>lock</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>apparent_power</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HA Lock</t>
+          <t>HA Sensor (apparent_power)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ha-lock-none</t>
+          <t>ha-sensor-apparent_power</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -9722,7 +9740,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>DOOR_OPEN</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -9732,7 +9750,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>ACCESS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -9742,7 +9760,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -9752,7 +9770,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>APPARENT_POWER</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -9762,13 +9780,31 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S50" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" t="n">
+        <v>10000</v>
+      </c>
+      <c r="U50" t="n">
+        <v>1</v>
+      </c>
+      <c r="V50" t="n">
+        <v>30</v>
+      </c>
+      <c r="W50" t="n">
+        <v>120</v>
+      </c>
+      <c r="X50" t="n">
+        <v>2</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -9782,7 +9818,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -9792,17 +9828,17 @@
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -9812,7 +9848,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH50" t="inlineStr">
@@ -9869,22 +9905,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>aqi</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HA Number</t>
+          <t>HA Sensor (aqi)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ha-number-none</t>
+          <t>ha-sensor-aqi</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -9939,23 +9975,41 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S51" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" t="n">
+        <v>500</v>
+      </c>
+      <c r="U51" t="n">
+        <v>1</v>
+      </c>
+      <c r="V51" t="n">
+        <v>30</v>
+      </c>
+      <c r="W51" t="n">
+        <v>120</v>
+      </c>
+      <c r="X51" t="n">
+        <v>2</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
@@ -9969,7 +10023,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>POSITIONAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -9979,27 +10033,27 @@
       </c>
       <c r="AC51" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>POWER_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH51" t="inlineStr">
@@ -10061,17 +10115,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>atmospheric_pressure</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>HA Sensor</t>
+          <t>HA Sensor (atmospheric_pressure)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ha-sensor-none</t>
+          <t>ha-sensor-atmospheric_pressure</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -10121,22 +10175,22 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>TEMPERATURE</t>
+          <t>AIR_PRESSURE</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -10145,10 +10199,10 @@
         </is>
       </c>
       <c r="S52" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="T52" t="n">
-        <v>100</v>
+        <v>1100</v>
       </c>
       <c r="U52" t="n">
         <v>0.1</v>
@@ -10164,7 +10218,7 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
@@ -10266,17 +10320,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>apparent_power</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HA Sensor (apparent_power)</t>
+          <t>HA Sensor (battery)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ha-sensor-apparent_power</t>
+          <t>ha-sensor-battery</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -10331,7 +10385,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>APPARENT_POWER</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -10353,16 +10407,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="U53" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V53" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="W53" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="X53" t="n">
         <v>2</v>
@@ -10471,17 +10525,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>aqi</t>
+          <t>carbon_dioxide</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HA Sensor (aqi)</t>
+          <t>HA Sensor (carbon_dioxide)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ha-sensor-aqi</t>
+          <t>ha-sensor-carbon_dioxide</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -10536,12 +10590,12 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>CO2_CONCENTRATION</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -10558,7 +10612,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="U54" t="n">
         <v>1</v>
@@ -10676,17 +10730,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>atmospheric_pressure</t>
+          <t>carbon_monoxide</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HA Sensor (atmospheric_pressure)</t>
+          <t>HA Sensor (carbon_monoxide)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ha-sensor-atmospheric_pressure</t>
+          <t>ha-sensor-carbon_monoxide</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -10741,7 +10795,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>AIR_PRESSURE</t>
+          <t>CO_CONCENTRATION</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -10751,7 +10805,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -10760,10 +10814,10 @@
         </is>
       </c>
       <c r="S55" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="U55" t="n">
         <v>0.1</v>
@@ -10881,17 +10935,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>current</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HA Sensor (battery)</t>
+          <t>HA Sensor (current)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ha-sensor-battery</t>
+          <t>ha-sensor-current</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -10946,7 +11000,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>ELECTRIC_CURRENT</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -10971,13 +11025,13 @@
         <v>100</v>
       </c>
       <c r="U56" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="V56" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="W56" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="X56" t="n">
         <v>2</v>
@@ -11086,17 +11140,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>carbon_dioxide</t>
+          <t>distance</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_dioxide)</t>
+          <t>HA Sensor (distance)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_dioxide</t>
+          <t>ha-sensor-distance</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -11151,17 +11205,17 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>CO2_CONCENTRATION</t>
+          <t>LENGTH</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -11173,10 +11227,10 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="U57" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="V57" t="n">
         <v>30</v>
@@ -11291,17 +11345,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>carbon_monoxide</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_monoxide)</t>
+          <t>HA Sensor (duration)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_monoxide</t>
+          <t>ha-sensor-duration</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -11356,17 +11410,17 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>CO_CONCENTRATION</t>
+          <t>DURATION</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -11378,10 +11432,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1000</v>
+        <v>86400</v>
       </c>
       <c r="U58" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="V58" t="n">
         <v>30</v>
@@ -11496,17 +11550,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>HA Sensor (current)</t>
+          <t>HA Sensor (energy)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ha-sensor-current</t>
+          <t>ha-sensor-energy</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -11561,7 +11615,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>ELECTRIC_CURRENT</t>
+          <t>ENERGY_METER</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -11583,10 +11637,10 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>100</v>
+        <v>100000</v>
       </c>
       <c r="U59" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="V59" t="n">
         <v>30</v>
@@ -11701,17 +11755,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>distance</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HA Sensor (distance)</t>
+          <t>HA Sensor (frequency)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ha-sensor-distance</t>
+          <t>ha-sensor-frequency</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -11766,12 +11820,12 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>FREQUENCY</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -11906,17 +11960,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>HA Sensor (duration)</t>
+          <t>HA Sensor (gas)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ha-sensor-duration</t>
+          <t>ha-sensor-gas</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -11966,12 +12020,12 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>DURATION</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -11981,7 +12035,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -11993,7 +12047,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>86400</v>
+        <v>100</v>
       </c>
       <c r="U61" t="n">
         <v>1</v>
@@ -12111,17 +12165,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>humidity</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HA Sensor (energy)</t>
+          <t>HA Sensor (humidity)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ha-sensor-energy</t>
+          <t>ha-sensor-humidity</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -12176,17 +12230,17 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>ENERGY_METER</t>
+          <t>HUMIDITY</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -12198,10 +12252,10 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>100000</v>
+        <v>100</v>
       </c>
       <c r="U62" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="V62" t="n">
         <v>30</v>
@@ -12316,17 +12370,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>illuminance</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>HA Sensor (frequency)</t>
+          <t>HA Sensor (illuminance)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ha-sensor-frequency</t>
+          <t>ha-sensor-illuminance</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -12381,17 +12435,17 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>FREQUENCY</t>
+          <t>ILLUMINATION</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -12403,10 +12457,10 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>1000</v>
+        <v>100000</v>
       </c>
       <c r="U63" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="V63" t="n">
         <v>30</v>
@@ -12521,17 +12575,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>moisture</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>HA Sensor (gas)</t>
+          <t>HA Sensor (moisture)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ha-sensor-gas</t>
+          <t>ha-sensor-moisture</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -12581,7 +12635,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -12611,7 +12665,7 @@
         <v>100</v>
       </c>
       <c r="U64" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V64" t="n">
         <v>30</v>
@@ -12726,17 +12780,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>humidity</t>
+          <t>pm1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HA Sensor (humidity)</t>
+          <t>HA Sensor (pm1)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ha-sensor-humidity</t>
+          <t>ha-sensor-pm1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -12791,17 +12845,17 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>HUMIDITY</t>
+          <t>PARTICLES_PM1</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -12813,10 +12867,10 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="U65" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V65" t="n">
         <v>30</v>
@@ -12931,17 +12985,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>illuminance</t>
+          <t>pm10</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>HA Sensor (illuminance)</t>
+          <t>HA Sensor (pm10)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ha-sensor-illuminance</t>
+          <t>ha-sensor-pm10</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -12996,17 +13050,17 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>ILLUMINATION</t>
+          <t>PARTICLES_PM10</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -13018,7 +13072,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>100000</v>
+        <v>500</v>
       </c>
       <c r="U66" t="n">
         <v>1</v>
@@ -13136,17 +13190,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>moisture</t>
+          <t>pm25</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HA Sensor (moisture)</t>
+          <t>HA Sensor (pm25)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ha-sensor-moisture</t>
+          <t>ha-sensor-pm25</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -13201,17 +13255,17 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PARTICLES_PM2_5</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -13223,10 +13277,10 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="U67" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V67" t="n">
         <v>30</v>
@@ -13341,17 +13395,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>pm1</t>
+          <t>power</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HA Sensor (pm1)</t>
+          <t>HA Sensor (power)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ha-sensor-pm1</t>
+          <t>ha-sensor-power</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -13406,7 +13460,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>PARTICLES_PM1</t>
+          <t>ACTIVE_POWER</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -13416,7 +13470,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -13428,7 +13482,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="U68" t="n">
         <v>1</v>
@@ -13546,17 +13600,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>pm10</t>
+          <t>power_factor</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HA Sensor (pm10)</t>
+          <t>HA Sensor (power_factor)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ha-sensor-pm10</t>
+          <t>ha-sensor-power_factor</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -13611,7 +13665,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>PARTICLES_PM10</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -13621,7 +13675,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -13633,10 +13687,10 @@
         <v>0</v>
       </c>
       <c r="T69" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="U69" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V69" t="n">
         <v>30</v>
@@ -13751,17 +13805,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>pm25</t>
+          <t>precipitation</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HA Sensor (pm25)</t>
+          <t>HA Sensor (precipitation)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ha-sensor-pm25</t>
+          <t>ha-sensor-precipitation</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -13816,7 +13870,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>PARTICLES_PM2_5</t>
+          <t>PRECIPITATION</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -13826,7 +13880,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -13838,10 +13892,10 @@
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="U70" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="V70" t="n">
         <v>30</v>
@@ -13956,17 +14010,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>power</t>
+          <t>sound_pressure</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HA Sensor (power)</t>
+          <t>HA Sensor (sound_pressure)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ha-sensor-power</t>
+          <t>ha-sensor-sound_pressure</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -14021,7 +14075,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>ACTIVE_POWER</t>
+          <t>SOUND_PRESSURE_LEVEL</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -14043,10 +14097,10 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>10000</v>
+        <v>130</v>
       </c>
       <c r="U71" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="V71" t="n">
         <v>30</v>
@@ -14161,17 +14215,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>power_factor</t>
+          <t>speed</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HA Sensor (power_factor)</t>
+          <t>HA Sensor (speed)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>ha-sensor-power_factor</t>
+          <t>ha-sensor-speed</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -14226,17 +14280,17 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -14248,10 +14302,10 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="U72" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="V72" t="n">
         <v>30</v>
@@ -14366,17 +14420,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>precipitation</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HA Sensor (precipitation)</t>
+          <t>HA Sensor (temperature)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ha-sensor-precipitation</t>
+          <t>ha-sensor-temperature</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -14431,17 +14485,17 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>PRECIPITATION</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -14450,10 +14504,10 @@
         </is>
       </c>
       <c r="S73" t="n">
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="T73" t="n">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="U73" t="n">
         <v>0.1</v>
@@ -14571,17 +14625,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>sound_pressure</t>
+          <t>voltage</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HA Sensor (sound_pressure)</t>
+          <t>HA Sensor (voltage)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ha-sensor-sound_pressure</t>
+          <t>ha-sensor-voltage</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -14636,7 +14690,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>SOUND_PRESSURE_LEVEL</t>
+          <t>SUPPLY_VOLTAGE</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -14658,7 +14712,7 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>130</v>
+        <v>500</v>
       </c>
       <c r="U74" t="n">
         <v>0.1</v>
@@ -14776,17 +14830,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>speed</t>
+          <t>water</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>HA Sensor (speed)</t>
+          <t>HA Sensor (water)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ha-sensor-speed</t>
+          <t>ha-sensor-water</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -14841,17 +14895,17 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>WATER_QUANTITY</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -14863,7 +14917,7 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>60</v>
+        <v>10000</v>
       </c>
       <c r="U75" t="n">
         <v>0.1</v>
@@ -14981,17 +15035,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HA Sensor (temperature)</t>
+          <t>HA Sensor (weight)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ha-sensor-temperature</t>
+          <t>ha-sensor-weight</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -15046,17 +15100,17 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>TEMPERATURE</t>
+          <t>MASS</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -15065,10 +15119,10 @@
         </is>
       </c>
       <c r="S76" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>85</v>
+        <v>1000</v>
       </c>
       <c r="U76" t="n">
         <v>0.1</v>
@@ -15186,17 +15240,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>voltage</t>
+          <t>wind_speed</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HA Sensor (voltage)</t>
+          <t>HA Sensor (wind_speed)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ha-sensor-voltage</t>
+          <t>ha-sensor-wind_speed</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -15246,12 +15300,12 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>SUPPLY_VOLTAGE</t>
+          <t>WIND_SPEED</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -15261,7 +15315,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -15273,7 +15327,7 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="U77" t="n">
         <v>0.1</v>
@@ -15386,22 +15440,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>siren</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HA Sensor (water)</t>
+          <t>HA Siren</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ha-sensor-water</t>
+          <t>ha-siren-none</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -15456,7 +15510,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>WATER_QUANTITY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -15466,67 +15520,49 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>CUSTOM</t>
+        </is>
+      </c>
+      <c r="AB78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S78" t="n">
-        <v>0</v>
-      </c>
-      <c r="T78" t="n">
-        <v>10000</v>
-      </c>
-      <c r="U78" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V78" t="n">
-        <v>30</v>
-      </c>
-      <c r="W78" t="n">
-        <v>120</v>
-      </c>
-      <c r="X78" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF78" t="inlineStr">
         <is>
           <t>no</t>
@@ -15534,12 +15570,12 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AUDIO_VOLUME</t>
         </is>
       </c>
       <c r="AI78" t="inlineStr">
@@ -15591,22 +15627,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>HA Sensor (weight)</t>
+          <t>HA Switch</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ha-sensor-weight</t>
+          <t>ha-switch-none</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -15661,7 +15697,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -15671,67 +15707,49 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S79" t="n">
-        <v>0</v>
-      </c>
-      <c r="T79" t="n">
-        <v>1000</v>
-      </c>
-      <c r="U79" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V79" t="n">
-        <v>30</v>
-      </c>
-      <c r="W79" t="n">
-        <v>120</v>
-      </c>
-      <c r="X79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF79" t="inlineStr">
         <is>
           <t>no</t>
@@ -15739,7 +15757,7 @@
       </c>
       <c r="AG79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH79" t="inlineStr">
@@ -15796,22 +15814,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>wind_speed</t>
+          <t>outlet</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HA Sensor (wind_speed)</t>
+          <t>HA Switch (outlet)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ha-sensor-wind_speed</t>
+          <t>ha-switch-outlet</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -15861,12 +15879,12 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>WIND_SPEED</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -15876,67 +15894,49 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S80" t="n">
-        <v>0</v>
-      </c>
-      <c r="T80" t="n">
-        <v>60</v>
-      </c>
-      <c r="U80" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V80" t="n">
-        <v>30</v>
-      </c>
-      <c r="W80" t="n">
-        <v>120</v>
-      </c>
-      <c r="X80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF80" t="inlineStr">
         <is>
           <t>no</t>
@@ -15944,7 +15944,7 @@
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH80" t="inlineStr">
@@ -16001,22 +16001,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>siren</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HA Siren</t>
+          <t>HA Switch (switch)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ha-siren-none</t>
+          <t>ha-switch-switch</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -16101,7 +16101,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>ON_OFF</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -16136,7 +16136,7 @@
       </c>
       <c r="AH81" t="inlineStr">
         <is>
-          <t>AUDIO_VOLUME</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI81" t="inlineStr">
@@ -16188,7 +16188,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>HA Switch</t>
+          <t>HA Valve</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>ha-switch-none</t>
+          <t>ha-valve-none</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -16218,7 +16218,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -16308,7 +16308,7 @@
       </c>
       <c r="AE82" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF82" t="inlineStr">
@@ -16375,22 +16375,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>outlet</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HA Switch (outlet)</t>
+          <t>HA Valve (gas)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ha-switch-outlet</t>
+          <t>ha-valve-gas</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="AE83" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF83" t="inlineStr">
@@ -16562,22 +16562,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>water</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>HA Switch (switch)</t>
+          <t>HA Valve (water)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ha-switch-switch</t>
+          <t>ha-valve-water</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -16662,7 +16662,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -16677,22 +16677,22 @@
       </c>
       <c r="AD84" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>GRADUAL</t>
         </is>
       </c>
       <c r="AE84" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>WATER_FLOW_RATE</t>
         </is>
       </c>
       <c r="AH84" t="inlineStr">
@@ -16754,17 +16754,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>water_heater</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>HA Valve</t>
+          <t>HA Valve (water_heater)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ha-valve-none</t>
+          <t>ha-valve-water_heater</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -16849,7 +16849,7 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="AD85" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>GRADUAL</t>
         </is>
       </c>
       <c r="AE85" t="inlineStr">
@@ -16874,12 +16874,12 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>WATER_FLOW_RATE</t>
         </is>
       </c>
       <c r="AH85" t="inlineStr">
@@ -16928,567 +16928,6 @@
         </is>
       </c>
       <c r="AQ85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>gas</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>HA Valve (gas)</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>ha-valve-gas</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA86" t="inlineStr">
-        <is>
-          <t>ON_OFF</t>
-        </is>
-      </c>
-      <c r="AB86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC86" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD86" t="inlineStr">
-        <is>
-          <t>BINARY</t>
-        </is>
-      </c>
-      <c r="AE86" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AG86" t="inlineStr">
-        <is>
-          <t>POWER_STATE</t>
-        </is>
-      </c>
-      <c r="AH86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>water</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>HA Valve (water)</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>ha-valve-water</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA87" t="inlineStr">
-        <is>
-          <t>POSITIONAL</t>
-        </is>
-      </c>
-      <c r="AB87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC87" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD87" t="inlineStr">
-        <is>
-          <t>GRADUAL</t>
-        </is>
-      </c>
-      <c r="AE87" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF87" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG87" t="inlineStr">
-        <is>
-          <t>WATER_FLOW_RATE</t>
-        </is>
-      </c>
-      <c r="AH87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>water_heater</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>HA Valve (water_heater)</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>ha-valve-water_heater</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA88" t="inlineStr">
-        <is>
-          <t>POSITIONAL</t>
-        </is>
-      </c>
-      <c r="AB88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC88" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD88" t="inlineStr">
-        <is>
-          <t>GRADUAL</t>
-        </is>
-      </c>
-      <c r="AE88" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF88" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG88" t="inlineStr">
-        <is>
-          <t>WATER_FLOW_RATE</t>
-        </is>
-      </c>
-      <c r="AH88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ88" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
revert: restore ha_vdsd_mapping.xlsx (not to be modified without explicit confirmation)
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ85"/>
+  <dimension ref="A1:AQ88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ha-light</t>
+          <t>ha-light-onoff</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -9121,22 +9121,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>lock</t>
+          <t>light</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>brightness</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HA Lock</t>
+          <t>HA Light (brightness)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ha-lock-none</t>
+          <t>ha-light-brightness</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -9151,7 +9151,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -9161,7 +9161,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>DOOR_OPEN</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>ACCESS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>DIMMER</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -9236,22 +9236,22 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>GRADUAL</t>
         </is>
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>LIGHTS</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>BRIGHTNESS</t>
         </is>
       </c>
       <c r="AH47" t="inlineStr">
@@ -9308,22 +9308,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>light</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>color_temp</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HA Number</t>
+          <t>HA Light (color_temp)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ha-number-none</t>
+          <t>ha-light-color_temp</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -9338,7 +9338,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>POSITIONAL</t>
+          <t>DIMMER_COLOR_TEMP</t>
         </is>
       </c>
       <c r="AB48" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>LIGHTS</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -9438,12 +9438,12 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>POWER_LEVEL</t>
+          <t>BRIGHTNESS</t>
         </is>
       </c>
       <c r="AH48" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>COLOR_TEMPERATURE</t>
         </is>
       </c>
       <c r="AI48" t="inlineStr">
@@ -9495,22 +9495,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>light</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rgb</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HA Sensor</t>
+          <t>HA Light (rgb)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ha-sensor-none</t>
+          <t>ha-light-rgb</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -9560,115 +9560,97 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>FULL_COLOR_DIMMER</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>GRADUAL</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>LIGHTS</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>TEMPERATURE</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>JOKER</t>
-        </is>
-      </c>
-      <c r="S49" t="n">
-        <v>0</v>
-      </c>
-      <c r="T49" t="n">
-        <v>100</v>
-      </c>
-      <c r="U49" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V49" t="n">
-        <v>30</v>
-      </c>
-      <c r="W49" t="n">
-        <v>120</v>
-      </c>
-      <c r="X49" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y49" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="Z49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BRIGHTNESS</t>
         </is>
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>HUE</t>
         </is>
       </c>
       <c r="AI49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SATURATION</t>
         </is>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>COLOR_TEMPERATURE</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIE_X</t>
         </is>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIE_Y</t>
         </is>
       </c>
       <c r="AM49" t="inlineStr">
@@ -9700,22 +9682,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>lock</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>apparent_power</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HA Sensor (apparent_power)</t>
+          <t>HA Lock</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ha-sensor-apparent_power</t>
+          <t>ha-lock-none</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -9740,7 +9722,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DOOR_OPEN</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -9750,7 +9732,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ACCESS</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -9760,7 +9742,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -9770,7 +9752,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>APPARENT_POWER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -9780,67 +9762,49 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>CUSTOM</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S50" t="n">
-        <v>0</v>
-      </c>
-      <c r="T50" t="n">
-        <v>10000</v>
-      </c>
-      <c r="U50" t="n">
-        <v>1</v>
-      </c>
-      <c r="V50" t="n">
-        <v>30</v>
-      </c>
-      <c r="W50" t="n">
-        <v>120</v>
-      </c>
-      <c r="X50" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z50" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB50" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF50" t="inlineStr">
         <is>
           <t>no</t>
@@ -9848,7 +9812,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH50" t="inlineStr">
@@ -9905,22 +9869,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>number</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>aqi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HA Sensor (aqi)</t>
+          <t>HA Number</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ha-sensor-aqi</t>
+          <t>ha-number-none</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -9975,85 +9939,67 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>POSITIONAL</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>GRADUAL</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>JOKER</t>
-        </is>
-      </c>
-      <c r="S51" t="n">
-        <v>0</v>
-      </c>
-      <c r="T51" t="n">
-        <v>500</v>
-      </c>
-      <c r="U51" t="n">
-        <v>1</v>
-      </c>
-      <c r="V51" t="n">
-        <v>30</v>
-      </c>
-      <c r="W51" t="n">
-        <v>120</v>
-      </c>
-      <c r="X51" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB51" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF51" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_LEVEL</t>
         </is>
       </c>
       <c r="AH51" t="inlineStr">
@@ -10115,17 +10061,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>atmospheric_pressure</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>HA Sensor (atmospheric_pressure)</t>
+          <t>HA Sensor</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ha-sensor-atmospheric_pressure</t>
+          <t>ha-sensor-none</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -10175,22 +10121,22 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>AIR_PRESSURE</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -10199,10 +10145,10 @@
         </is>
       </c>
       <c r="S52" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>1100</v>
+        <v>100</v>
       </c>
       <c r="U52" t="n">
         <v>0.1</v>
@@ -10218,7 +10164,7 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
@@ -10320,17 +10266,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>apparent_power</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HA Sensor (battery)</t>
+          <t>HA Sensor (apparent_power)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ha-sensor-battery</t>
+          <t>ha-sensor-apparent_power</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -10385,7 +10331,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>APPARENT_POWER</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -10407,16 +10353,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>100</v>
+        <v>10000</v>
       </c>
       <c r="U53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V53" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="W53" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="X53" t="n">
         <v>2</v>
@@ -10525,17 +10471,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>carbon_dioxide</t>
+          <t>aqi</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_dioxide)</t>
+          <t>HA Sensor (aqi)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_dioxide</t>
+          <t>ha-sensor-aqi</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -10590,12 +10536,12 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>CO2_CONCENTRATION</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -10612,7 +10558,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>5000</v>
+        <v>500</v>
       </c>
       <c r="U54" t="n">
         <v>1</v>
@@ -10730,17 +10676,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>carbon_monoxide</t>
+          <t>atmospheric_pressure</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_monoxide)</t>
+          <t>HA Sensor (atmospheric_pressure)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_monoxide</t>
+          <t>ha-sensor-atmospheric_pressure</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -10795,7 +10741,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>CO_CONCENTRATION</t>
+          <t>AIR_PRESSURE</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -10805,7 +10751,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -10814,10 +10760,10 @@
         </is>
       </c>
       <c r="S55" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="T55" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="U55" t="n">
         <v>0.1</v>
@@ -10935,17 +10881,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HA Sensor (current)</t>
+          <t>HA Sensor (battery)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ha-sensor-current</t>
+          <t>ha-sensor-battery</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -11000,7 +10946,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>ELECTRIC_CURRENT</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -11025,13 +10971,13 @@
         <v>100</v>
       </c>
       <c r="U56" t="n">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="V56" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="W56" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="X56" t="n">
         <v>2</v>
@@ -11140,17 +11086,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>distance</t>
+          <t>carbon_dioxide</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HA Sensor (distance)</t>
+          <t>HA Sensor (carbon_dioxide)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ha-sensor-distance</t>
+          <t>ha-sensor-carbon_dioxide</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -11205,17 +11151,17 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>CO2_CONCENTRATION</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -11227,10 +11173,10 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="U57" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="V57" t="n">
         <v>30</v>
@@ -11345,17 +11291,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>carbon_monoxide</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HA Sensor (duration)</t>
+          <t>HA Sensor (carbon_monoxide)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ha-sensor-duration</t>
+          <t>ha-sensor-carbon_monoxide</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -11410,17 +11356,17 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>DURATION</t>
+          <t>CO_CONCENTRATION</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -11432,10 +11378,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>86400</v>
+        <v>1000</v>
       </c>
       <c r="U58" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="V58" t="n">
         <v>30</v>
@@ -11550,17 +11496,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>current</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>HA Sensor (energy)</t>
+          <t>HA Sensor (current)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ha-sensor-energy</t>
+          <t>ha-sensor-current</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -11615,7 +11561,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>ENERGY_METER</t>
+          <t>ELECTRIC_CURRENT</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -11637,10 +11583,10 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>100000</v>
+        <v>100</v>
       </c>
       <c r="U59" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="V59" t="n">
         <v>30</v>
@@ -11755,17 +11701,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>distance</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HA Sensor (frequency)</t>
+          <t>HA Sensor (distance)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ha-sensor-frequency</t>
+          <t>ha-sensor-distance</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -11820,12 +11766,12 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>FREQUENCY</t>
+          <t>LENGTH</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -11960,17 +11906,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>HA Sensor (gas)</t>
+          <t>HA Sensor (duration)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ha-sensor-gas</t>
+          <t>ha-sensor-duration</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -12020,22 +11966,22 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>DURATION</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -12047,7 +11993,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>100</v>
+        <v>86400</v>
       </c>
       <c r="U61" t="n">
         <v>1</v>
@@ -12165,17 +12111,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>humidity</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HA Sensor (humidity)</t>
+          <t>HA Sensor (energy)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ha-sensor-humidity</t>
+          <t>ha-sensor-energy</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -12230,17 +12176,17 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>HUMIDITY</t>
+          <t>ENERGY_METER</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -12252,10 +12198,10 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>100</v>
+        <v>100000</v>
       </c>
       <c r="U62" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="V62" t="n">
         <v>30</v>
@@ -12370,17 +12316,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>illuminance</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>HA Sensor (illuminance)</t>
+          <t>HA Sensor (frequency)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ha-sensor-illuminance</t>
+          <t>ha-sensor-frequency</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -12435,17 +12381,17 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>ILLUMINATION</t>
+          <t>FREQUENCY</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -12457,10 +12403,10 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>100000</v>
+        <v>1000</v>
       </c>
       <c r="U63" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="V63" t="n">
         <v>30</v>
@@ -12575,17 +12521,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>moisture</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>HA Sensor (moisture)</t>
+          <t>HA Sensor (gas)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ha-sensor-moisture</t>
+          <t>ha-sensor-gas</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -12635,7 +12581,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -12665,7 +12611,7 @@
         <v>100</v>
       </c>
       <c r="U64" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V64" t="n">
         <v>30</v>
@@ -12780,17 +12726,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>pm1</t>
+          <t>humidity</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HA Sensor (pm1)</t>
+          <t>HA Sensor (humidity)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ha-sensor-pm1</t>
+          <t>ha-sensor-humidity</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -12845,17 +12791,17 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>PARTICLES_PM1</t>
+          <t>HUMIDITY</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -12867,10 +12813,10 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="U65" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V65" t="n">
         <v>30</v>
@@ -12985,17 +12931,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>pm10</t>
+          <t>illuminance</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>HA Sensor (pm10)</t>
+          <t>HA Sensor (illuminance)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ha-sensor-pm10</t>
+          <t>ha-sensor-illuminance</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -13050,17 +12996,17 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>PARTICLES_PM10</t>
+          <t>ILLUMINATION</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -13072,7 +13018,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>500</v>
+        <v>100000</v>
       </c>
       <c r="U66" t="n">
         <v>1</v>
@@ -13190,17 +13136,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>pm25</t>
+          <t>moisture</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HA Sensor (pm25)</t>
+          <t>HA Sensor (moisture)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ha-sensor-pm25</t>
+          <t>ha-sensor-moisture</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -13255,17 +13201,17 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>PARTICLES_PM2_5</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -13277,10 +13223,10 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="U67" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V67" t="n">
         <v>30</v>
@@ -13395,17 +13341,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>power</t>
+          <t>pm1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HA Sensor (power)</t>
+          <t>HA Sensor (pm1)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ha-sensor-power</t>
+          <t>ha-sensor-pm1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -13460,7 +13406,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>ACTIVE_POWER</t>
+          <t>PARTICLES_PM1</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -13470,7 +13416,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -13482,7 +13428,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="U68" t="n">
         <v>1</v>
@@ -13600,17 +13546,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>power_factor</t>
+          <t>pm10</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HA Sensor (power_factor)</t>
+          <t>HA Sensor (pm10)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ha-sensor-power_factor</t>
+          <t>ha-sensor-pm10</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -13665,7 +13611,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>PARTICLES_PM10</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -13675,7 +13621,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -13687,10 +13633,10 @@
         <v>0</v>
       </c>
       <c r="T69" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="U69" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V69" t="n">
         <v>30</v>
@@ -13805,17 +13751,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>precipitation</t>
+          <t>pm25</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HA Sensor (precipitation)</t>
+          <t>HA Sensor (pm25)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ha-sensor-precipitation</t>
+          <t>ha-sensor-pm25</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -13870,7 +13816,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>PRECIPITATION</t>
+          <t>PARTICLES_PM2_5</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -13880,7 +13826,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -13892,10 +13838,10 @@
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="U70" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="V70" t="n">
         <v>30</v>
@@ -14010,17 +13956,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>sound_pressure</t>
+          <t>power</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HA Sensor (sound_pressure)</t>
+          <t>HA Sensor (power)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ha-sensor-sound_pressure</t>
+          <t>ha-sensor-power</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -14075,7 +14021,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>SOUND_PRESSURE_LEVEL</t>
+          <t>ACTIVE_POWER</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -14097,10 +14043,10 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>130</v>
+        <v>10000</v>
       </c>
       <c r="U71" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="V71" t="n">
         <v>30</v>
@@ -14215,17 +14161,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>speed</t>
+          <t>power_factor</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HA Sensor (speed)</t>
+          <t>HA Sensor (power_factor)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>ha-sensor-speed</t>
+          <t>ha-sensor-power_factor</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -14280,17 +14226,17 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -14302,10 +14248,10 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="U72" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="V72" t="n">
         <v>30</v>
@@ -14420,17 +14366,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>precipitation</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HA Sensor (temperature)</t>
+          <t>HA Sensor (precipitation)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ha-sensor-temperature</t>
+          <t>ha-sensor-precipitation</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -14485,17 +14431,17 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>TEMPERATURE</t>
+          <t>PRECIPITATION</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -14504,10 +14450,10 @@
         </is>
       </c>
       <c r="S73" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="T73" t="n">
-        <v>85</v>
+        <v>200</v>
       </c>
       <c r="U73" t="n">
         <v>0.1</v>
@@ -14625,17 +14571,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>voltage</t>
+          <t>sound_pressure</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HA Sensor (voltage)</t>
+          <t>HA Sensor (sound_pressure)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ha-sensor-voltage</t>
+          <t>ha-sensor-sound_pressure</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -14690,7 +14636,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>SUPPLY_VOLTAGE</t>
+          <t>SOUND_PRESSURE_LEVEL</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -14712,7 +14658,7 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>500</v>
+        <v>130</v>
       </c>
       <c r="U74" t="n">
         <v>0.1</v>
@@ -14830,17 +14776,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>speed</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>HA Sensor (water)</t>
+          <t>HA Sensor (speed)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ha-sensor-water</t>
+          <t>ha-sensor-speed</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -14895,17 +14841,17 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>WATER_QUANTITY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -14917,7 +14863,7 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>10000</v>
+        <v>60</v>
       </c>
       <c r="U75" t="n">
         <v>0.1</v>
@@ -15035,17 +14981,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HA Sensor (weight)</t>
+          <t>HA Sensor (temperature)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ha-sensor-weight</t>
+          <t>ha-sensor-temperature</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -15100,17 +15046,17 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -15119,10 +15065,10 @@
         </is>
       </c>
       <c r="S76" t="n">
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="T76" t="n">
-        <v>1000</v>
+        <v>85</v>
       </c>
       <c r="U76" t="n">
         <v>0.1</v>
@@ -15240,17 +15186,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>wind_speed</t>
+          <t>voltage</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HA Sensor (wind_speed)</t>
+          <t>HA Sensor (voltage)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ha-sensor-wind_speed</t>
+          <t>ha-sensor-voltage</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -15300,12 +15246,12 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>WIND_SPEED</t>
+          <t>SUPPLY_VOLTAGE</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -15315,7 +15261,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -15327,7 +15273,7 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>60</v>
+        <v>500</v>
       </c>
       <c r="U77" t="n">
         <v>0.1</v>
@@ -15440,22 +15386,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>siren</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>water</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HA Siren</t>
+          <t>HA Sensor (water)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ha-siren-none</t>
+          <t>ha-sensor-water</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -15510,7 +15456,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>WATER_QUANTITY</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -15520,13 +15466,31 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" t="n">
+        <v>10000</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V78" t="n">
+        <v>30</v>
+      </c>
+      <c r="W78" t="n">
+        <v>120</v>
+      </c>
+      <c r="X78" t="n">
+        <v>2</v>
       </c>
       <c r="Y78" t="inlineStr">
         <is>
@@ -15540,7 +15504,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -15550,17 +15514,17 @@
       </c>
       <c r="AC78" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD78" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE78" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF78" t="inlineStr">
@@ -15570,12 +15534,12 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH78" t="inlineStr">
         <is>
-          <t>AUDIO_VOLUME</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI78" t="inlineStr">
@@ -15627,22 +15591,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>HA Switch</t>
+          <t>HA Sensor (weight)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ha-switch-none</t>
+          <t>ha-sensor-weight</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -15697,7 +15661,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MASS</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -15707,13 +15671,31 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S79" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V79" t="n">
+        <v>30</v>
+      </c>
+      <c r="W79" t="n">
+        <v>120</v>
+      </c>
+      <c r="X79" t="n">
+        <v>2</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -15727,7 +15709,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -15737,17 +15719,17 @@
       </c>
       <c r="AC79" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD79" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE79" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF79" t="inlineStr">
@@ -15757,7 +15739,7 @@
       </c>
       <c r="AG79" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH79" t="inlineStr">
@@ -15814,22 +15796,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>outlet</t>
+          <t>wind_speed</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HA Switch (outlet)</t>
+          <t>HA Sensor (wind_speed)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ha-switch-outlet</t>
+          <t>ha-sensor-wind_speed</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -15879,12 +15861,12 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>WIND_SPEED</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -15894,13 +15876,31 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S80" t="n">
+        <v>0</v>
+      </c>
+      <c r="T80" t="n">
+        <v>60</v>
+      </c>
+      <c r="U80" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V80" t="n">
+        <v>30</v>
+      </c>
+      <c r="W80" t="n">
+        <v>120</v>
+      </c>
+      <c r="X80" t="n">
+        <v>2</v>
       </c>
       <c r="Y80" t="inlineStr">
         <is>
@@ -15914,7 +15914,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -15924,17 +15924,17 @@
       </c>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD80" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE80" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF80" t="inlineStr">
@@ -15944,7 +15944,7 @@
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH80" t="inlineStr">
@@ -16001,22 +16001,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>siren</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HA Switch (switch)</t>
+          <t>HA Siren</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ha-switch-switch</t>
+          <t>ha-siren-none</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -16101,7 +16101,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -16136,7 +16136,7 @@
       </c>
       <c r="AH81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AUDIO_VOLUME</t>
         </is>
       </c>
       <c r="AI81" t="inlineStr">
@@ -16188,7 +16188,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>valve</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -16198,12 +16198,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>HA Valve</t>
+          <t>HA Switch</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>ha-valve-none</t>
+          <t>ha-switch-none</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -16218,7 +16218,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -16308,7 +16308,7 @@
       </c>
       <c r="AE82" t="inlineStr">
         <is>
-          <t>HEATING</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF82" t="inlineStr">
@@ -16375,22 +16375,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>valve</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>outlet</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HA Valve (gas)</t>
+          <t>HA Switch (outlet)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ha-valve-gas</t>
+          <t>ha-switch-outlet</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="AE83" t="inlineStr">
         <is>
-          <t>HEATING</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF83" t="inlineStr">
@@ -16562,22 +16562,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>valve</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>HA Valve (water)</t>
+          <t>HA Switch (switch)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ha-valve-water</t>
+          <t>ha-switch-switch</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -16662,7 +16662,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>POSITIONAL</t>
+          <t>ON_OFF</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -16677,22 +16677,22 @@
       </c>
       <c r="AD84" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>BINARY</t>
         </is>
       </c>
       <c r="AE84" t="inlineStr">
         <is>
-          <t>HEATING</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>WATER_FLOW_RATE</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH84" t="inlineStr">
@@ -16754,180 +16754,741 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>HA Valve</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ha-valve-none</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Home Assistant</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC85" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE85" t="inlineStr">
+        <is>
+          <t>HEATING</t>
+        </is>
+      </c>
+      <c r="AF85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AG85" t="inlineStr">
+        <is>
+          <t>POWER_STATE</t>
+        </is>
+      </c>
+      <c r="AH85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AO85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>valve</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>gas</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>HA Valve (gas)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ha-valve-gas</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Home Assistant</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC86" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE86" t="inlineStr">
+        <is>
+          <t>HEATING</t>
+        </is>
+      </c>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AG86" t="inlineStr">
+        <is>
+          <t>POWER_STATE</t>
+        </is>
+      </c>
+      <c r="AH86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AO86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>valve</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>HA Valve (water)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ha-valve-water</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Home Assistant</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>BLUE</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>POSITIONAL</t>
+        </is>
+      </c>
+      <c r="AB87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>GRADUAL</t>
+        </is>
+      </c>
+      <c r="AE87" t="inlineStr">
+        <is>
+          <t>HEATING</t>
+        </is>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG87" t="inlineStr">
+        <is>
+          <t>WATER_FLOW_RATE</t>
+        </is>
+      </c>
+      <c r="AH87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AO87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>valve</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>water_heater</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>HA Valve (water_heater)</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>ha-valve-water_heater</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>Home Assistant</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
         <is>
           <t>BLUE</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA85" t="inlineStr">
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
         <is>
           <t>POSITIONAL</t>
         </is>
       </c>
-      <c r="AB85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC85" t="inlineStr">
+      <c r="AB88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC88" t="inlineStr">
         <is>
           <t>ROOM</t>
         </is>
       </c>
-      <c r="AD85" t="inlineStr">
+      <c r="AD88" t="inlineStr">
         <is>
           <t>GRADUAL</t>
         </is>
       </c>
-      <c r="AE85" t="inlineStr">
+      <c r="AE88" t="inlineStr">
         <is>
           <t>HEATING</t>
         </is>
       </c>
-      <c r="AF85" t="inlineStr">
+      <c r="AF88" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AG85" t="inlineStr">
+      <c r="AG88" t="inlineStr">
         <is>
           <t>WATER_FLOW_RATE</t>
         </is>
       </c>
-      <c r="AH85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ85" t="inlineStr">
+      <c r="AH88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AI88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AK88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AL88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AO88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ88" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
docs: update ha_vdsd_mapping.xlsx for light derive_fn refactor (approved)
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_lookups" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Mapping" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_lookups" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ88"/>
+  <dimension ref="A1:AQ85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ha-light-onoff</t>
+          <t>ha-light</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -9025,71 +9025,6 @@
       <c r="Y46" t="inlineStr">
         <is>
           <t>no</t>
-        </is>
-      </c>
-      <c r="Z46" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA46" t="inlineStr">
-        <is>
-          <t>ON_OFF</t>
-        </is>
-      </c>
-      <c r="AB46" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC46" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD46" t="inlineStr">
-        <is>
-          <t>BINARY</t>
-        </is>
-      </c>
-      <c r="AE46" t="inlineStr">
-        <is>
-          <t>LIGHTS</t>
-        </is>
-      </c>
-      <c r="AF46" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG46" t="inlineStr">
-        <is>
-          <t>BRIGHTNESS</t>
-        </is>
-      </c>
-      <c r="AH46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL46" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="AM46" t="inlineStr">
@@ -9121,22 +9056,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>lock</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>brightness</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HA Light (brightness)</t>
+          <t>HA Lock</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ha-light-brightness</t>
+          <t>ha-lock-none</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -9151,7 +9086,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -9161,7 +9096,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DOOR_OPEN</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -9171,7 +9106,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ACCESS</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -9181,7 +9116,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -9221,7 +9156,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>DIMMER</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -9236,22 +9171,22 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>BINARY</t>
         </is>
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH47" t="inlineStr">
@@ -9308,22 +9243,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>number</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>color_temp</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HA Light (color_temp)</t>
+          <t>HA Number</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ha-light-color_temp</t>
+          <t>ha-number-none</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -9338,7 +9273,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -9408,7 +9343,7 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>DIMMER_COLOR_TEMP</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB48" t="inlineStr">
@@ -9428,7 +9363,7 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>JOKER</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -9438,12 +9373,12 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>POWER_LEVEL</t>
         </is>
       </c>
       <c r="AH48" t="inlineStr">
         <is>
-          <t>COLOR_TEMPERATURE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI48" t="inlineStr">
@@ -9495,22 +9430,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>rgb</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HA Light (rgb)</t>
+          <t>HA Sensor</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ha-light-rgb</t>
+          <t>ha-sensor-none</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -9525,7 +9460,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -9560,32 +9495,50 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>100</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V49" t="n">
+        <v>30</v>
+      </c>
+      <c r="W49" t="n">
+        <v>120</v>
+      </c>
+      <c r="X49" t="n">
+        <v>2</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr">
@@ -9595,7 +9548,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>FULL_COLOR_DIMMER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -9605,52 +9558,52 @@
       </c>
       <c r="AC49" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>LIGHTS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>BRIGHTNESS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>HUE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI49" t="inlineStr">
         <is>
-          <t>SATURATION</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>COLOR_TEMPERATURE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>CIE_X</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
-          <t>CIE_Y</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AM49" t="inlineStr">
@@ -9682,22 +9635,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>lock</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>apparent_power</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>HA Lock</t>
+          <t>HA Sensor (apparent_power)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ha-lock-none</t>
+          <t>ha-sensor-apparent_power</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -9722,7 +9675,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>DOOR_OPEN</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -9732,7 +9685,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>ACCESS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -9742,7 +9695,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -9752,7 +9705,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>APPARENT_POWER</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -9762,13 +9715,31 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S50" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" t="n">
+        <v>10000</v>
+      </c>
+      <c r="U50" t="n">
+        <v>1</v>
+      </c>
+      <c r="V50" t="n">
+        <v>30</v>
+      </c>
+      <c r="W50" t="n">
+        <v>120</v>
+      </c>
+      <c r="X50" t="n">
+        <v>2</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -9782,7 +9753,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -9792,17 +9763,17 @@
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -9812,7 +9783,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH50" t="inlineStr">
@@ -9869,22 +9840,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>sensor</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>aqi</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HA Number</t>
+          <t>HA Sensor (aqi)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ha-number-none</t>
+          <t>ha-sensor-aqi</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -9939,23 +9910,41 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
+          <t>JOKER</t>
+        </is>
+      </c>
+      <c r="S51" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" t="n">
+        <v>500</v>
+      </c>
+      <c r="U51" t="n">
+        <v>1</v>
+      </c>
+      <c r="V51" t="n">
+        <v>30</v>
+      </c>
+      <c r="W51" t="n">
+        <v>120</v>
+      </c>
+      <c r="X51" t="n">
+        <v>2</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
@@ -9969,7 +9958,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>POSITIONAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -9979,27 +9968,27 @@
       </c>
       <c r="AC51" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>GRADUAL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>POWER_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AH51" t="inlineStr">
@@ -10061,17 +10050,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>atmospheric_pressure</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>HA Sensor</t>
+          <t>HA Sensor (atmospheric_pressure)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ha-sensor-none</t>
+          <t>ha-sensor-atmospheric_pressure</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -10121,22 +10110,22 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>TEMPERATURE</t>
+          <t>AIR_PRESSURE</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -10145,10 +10134,10 @@
         </is>
       </c>
       <c r="S52" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="T52" t="n">
-        <v>100</v>
+        <v>1100</v>
       </c>
       <c r="U52" t="n">
         <v>0.1</v>
@@ -10164,7 +10153,7 @@
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
@@ -10266,17 +10255,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>apparent_power</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HA Sensor (apparent_power)</t>
+          <t>HA Sensor (battery)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ha-sensor-apparent_power</t>
+          <t>ha-sensor-battery</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -10331,7 +10320,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>APPARENT_POWER</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -10353,16 +10342,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="U53" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V53" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="W53" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="X53" t="n">
         <v>2</v>
@@ -10471,17 +10460,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>aqi</t>
+          <t>carbon_dioxide</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HA Sensor (aqi)</t>
+          <t>HA Sensor (carbon_dioxide)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ha-sensor-aqi</t>
+          <t>ha-sensor-carbon_dioxide</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -10536,12 +10525,12 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>CO2_CONCENTRATION</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -10558,7 +10547,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="U54" t="n">
         <v>1</v>
@@ -10676,17 +10665,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>atmospheric_pressure</t>
+          <t>carbon_monoxide</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HA Sensor (atmospheric_pressure)</t>
+          <t>HA Sensor (carbon_monoxide)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ha-sensor-atmospheric_pressure</t>
+          <t>ha-sensor-carbon_monoxide</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -10741,7 +10730,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>AIR_PRESSURE</t>
+          <t>CO_CONCENTRATION</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -10751,7 +10740,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -10760,10 +10749,10 @@
         </is>
       </c>
       <c r="S55" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="U55" t="n">
         <v>0.1</v>
@@ -10881,17 +10870,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>current</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HA Sensor (battery)</t>
+          <t>HA Sensor (current)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ha-sensor-battery</t>
+          <t>ha-sensor-current</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -10946,7 +10935,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>ELECTRIC_CURRENT</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -10971,13 +10960,13 @@
         <v>100</v>
       </c>
       <c r="U56" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="V56" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="W56" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="X56" t="n">
         <v>2</v>
@@ -11086,17 +11075,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>carbon_dioxide</t>
+          <t>distance</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_dioxide)</t>
+          <t>HA Sensor (distance)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_dioxide</t>
+          <t>ha-sensor-distance</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -11151,17 +11140,17 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>CO2_CONCENTRATION</t>
+          <t>LENGTH</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -11173,10 +11162,10 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="U57" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="V57" t="n">
         <v>30</v>
@@ -11291,17 +11280,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>carbon_monoxide</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HA Sensor (carbon_monoxide)</t>
+          <t>HA Sensor (duration)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ha-sensor-carbon_monoxide</t>
+          <t>ha-sensor-duration</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -11356,17 +11345,17 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>CO_CONCENTRATION</t>
+          <t>DURATION</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -11378,10 +11367,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1000</v>
+        <v>86400</v>
       </c>
       <c r="U58" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="V58" t="n">
         <v>30</v>
@@ -11496,17 +11485,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>HA Sensor (current)</t>
+          <t>HA Sensor (energy)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ha-sensor-current</t>
+          <t>ha-sensor-energy</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -11561,7 +11550,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>ELECTRIC_CURRENT</t>
+          <t>ENERGY_METER</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -11583,10 +11572,10 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>100</v>
+        <v>100000</v>
       </c>
       <c r="U59" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="V59" t="n">
         <v>30</v>
@@ -11701,17 +11690,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>distance</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HA Sensor (distance)</t>
+          <t>HA Sensor (frequency)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ha-sensor-distance</t>
+          <t>ha-sensor-frequency</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -11766,12 +11755,12 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>FREQUENCY</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -11906,17 +11895,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>HA Sensor (duration)</t>
+          <t>HA Sensor (gas)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ha-sensor-duration</t>
+          <t>ha-sensor-gas</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -11966,12 +11955,12 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>DURATION</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -11981,7 +11970,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -11993,7 +11982,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>86400</v>
+        <v>100</v>
       </c>
       <c r="U61" t="n">
         <v>1</v>
@@ -12111,17 +12100,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>humidity</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HA Sensor (energy)</t>
+          <t>HA Sensor (humidity)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ha-sensor-energy</t>
+          <t>ha-sensor-humidity</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -12176,17 +12165,17 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>ENERGY_METER</t>
+          <t>HUMIDITY</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -12198,10 +12187,10 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>100000</v>
+        <v>100</v>
       </c>
       <c r="U62" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="V62" t="n">
         <v>30</v>
@@ -12316,17 +12305,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>illuminance</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>HA Sensor (frequency)</t>
+          <t>HA Sensor (illuminance)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ha-sensor-frequency</t>
+          <t>ha-sensor-illuminance</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -12381,17 +12370,17 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>FREQUENCY</t>
+          <t>ILLUMINATION</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -12403,10 +12392,10 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>1000</v>
+        <v>100000</v>
       </c>
       <c r="U63" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="V63" t="n">
         <v>30</v>
@@ -12521,17 +12510,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>moisture</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>HA Sensor (gas)</t>
+          <t>HA Sensor (moisture)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ha-sensor-gas</t>
+          <t>ha-sensor-moisture</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -12581,7 +12570,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -12611,7 +12600,7 @@
         <v>100</v>
       </c>
       <c r="U64" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V64" t="n">
         <v>30</v>
@@ -12726,17 +12715,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>humidity</t>
+          <t>pm1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HA Sensor (humidity)</t>
+          <t>HA Sensor (pm1)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ha-sensor-humidity</t>
+          <t>ha-sensor-pm1</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -12791,17 +12780,17 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>HUMIDITY</t>
+          <t>PARTICLES_PM1</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -12813,10 +12802,10 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="U65" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V65" t="n">
         <v>30</v>
@@ -12931,17 +12920,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>illuminance</t>
+          <t>pm10</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>HA Sensor (illuminance)</t>
+          <t>HA Sensor (pm10)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ha-sensor-illuminance</t>
+          <t>ha-sensor-pm10</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -12996,17 +12985,17 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>ILLUMINATION</t>
+          <t>PARTICLES_PM10</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -13018,7 +13007,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>100000</v>
+        <v>500</v>
       </c>
       <c r="U66" t="n">
         <v>1</v>
@@ -13136,17 +13125,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>moisture</t>
+          <t>pm25</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HA Sensor (moisture)</t>
+          <t>HA Sensor (pm25)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ha-sensor-moisture</t>
+          <t>ha-sensor-pm25</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -13201,17 +13190,17 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PARTICLES_PM2_5</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>ROOM</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -13223,10 +13212,10 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="U67" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="V67" t="n">
         <v>30</v>
@@ -13341,17 +13330,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>pm1</t>
+          <t>power</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HA Sensor (pm1)</t>
+          <t>HA Sensor (power)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ha-sensor-pm1</t>
+          <t>ha-sensor-power</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -13406,7 +13395,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>PARTICLES_PM1</t>
+          <t>ACTIVE_POWER</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -13416,7 +13405,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -13428,7 +13417,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="U68" t="n">
         <v>1</v>
@@ -13546,17 +13535,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>pm10</t>
+          <t>power_factor</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HA Sensor (pm10)</t>
+          <t>HA Sensor (power_factor)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ha-sensor-pm10</t>
+          <t>ha-sensor-power_factor</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -13611,7 +13600,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>PARTICLES_PM10</t>
+          <t>PERCENT</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -13621,7 +13610,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -13633,10 +13622,10 @@
         <v>0</v>
       </c>
       <c r="T69" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="U69" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="V69" t="n">
         <v>30</v>
@@ -13751,17 +13740,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>pm25</t>
+          <t>precipitation</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HA Sensor (pm25)</t>
+          <t>HA Sensor (precipitation)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ha-sensor-pm25</t>
+          <t>ha-sensor-precipitation</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -13816,7 +13805,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>PARTICLES_PM2_5</t>
+          <t>PRECIPITATION</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -13826,7 +13815,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>ROOM</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -13838,10 +13827,10 @@
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="U70" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="V70" t="n">
         <v>30</v>
@@ -13956,17 +13945,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>power</t>
+          <t>sound_pressure</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HA Sensor (power)</t>
+          <t>HA Sensor (sound_pressure)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>ha-sensor-power</t>
+          <t>ha-sensor-sound_pressure</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -14021,7 +14010,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>ACTIVE_POWER</t>
+          <t>SOUND_PRESSURE_LEVEL</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -14043,10 +14032,10 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>10000</v>
+        <v>130</v>
       </c>
       <c r="U71" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="V71" t="n">
         <v>30</v>
@@ -14161,17 +14150,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>power_factor</t>
+          <t>speed</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HA Sensor (power_factor)</t>
+          <t>HA Sensor (speed)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>ha-sensor-power_factor</t>
+          <t>ha-sensor-speed</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -14226,17 +14215,17 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>PERCENT</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -14248,10 +14237,10 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="U72" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="V72" t="n">
         <v>30</v>
@@ -14366,17 +14355,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>precipitation</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HA Sensor (precipitation)</t>
+          <t>HA Sensor (temperature)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ha-sensor-precipitation</t>
+          <t>ha-sensor-temperature</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -14431,17 +14420,17 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>PRECIPITATION</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>UNDEFINED</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -14450,10 +14439,10 @@
         </is>
       </c>
       <c r="S73" t="n">
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="T73" t="n">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="U73" t="n">
         <v>0.1</v>
@@ -14571,17 +14560,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>sound_pressure</t>
+          <t>voltage</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HA Sensor (sound_pressure)</t>
+          <t>HA Sensor (voltage)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ha-sensor-sound_pressure</t>
+          <t>ha-sensor-voltage</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -14636,7 +14625,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>SOUND_PRESSURE_LEVEL</t>
+          <t>SUPPLY_VOLTAGE</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -14658,7 +14647,7 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>130</v>
+        <v>500</v>
       </c>
       <c r="U74" t="n">
         <v>0.1</v>
@@ -14776,17 +14765,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>speed</t>
+          <t>water</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>HA Sensor (speed)</t>
+          <t>HA Sensor (water)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ha-sensor-speed</t>
+          <t>ha-sensor-water</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -14841,17 +14830,17 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>WATER_QUANTITY</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -14863,7 +14852,7 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>60</v>
+        <v>10000</v>
       </c>
       <c r="U75" t="n">
         <v>0.1</v>
@@ -14981,17 +14970,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HA Sensor (temperature)</t>
+          <t>HA Sensor (weight)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ha-sensor-temperature</t>
+          <t>ha-sensor-weight</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -15046,17 +15035,17 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>TEMPERATURE</t>
+          <t>MASS</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>UNDEFINED</t>
+          <t>DEVICE_LEVEL</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -15065,10 +15054,10 @@
         </is>
       </c>
       <c r="S76" t="n">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>85</v>
+        <v>1000</v>
       </c>
       <c r="U76" t="n">
         <v>0.1</v>
@@ -15186,17 +15175,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>voltage</t>
+          <t>wind_speed</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HA Sensor (voltage)</t>
+          <t>HA Sensor (wind_speed)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ha-sensor-voltage</t>
+          <t>ha-sensor-wind_speed</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -15246,12 +15235,12 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>SUPPLY_VOLTAGE</t>
+          <t>WIND_SPEED</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -15261,7 +15250,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>OUTDOOR</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -15273,7 +15262,7 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="U77" t="n">
         <v>0.1</v>
@@ -15386,22 +15375,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>siren</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HA Sensor (water)</t>
+          <t>HA Siren</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ha-sensor-water</t>
+          <t>ha-siren-none</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -15456,7 +15445,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>WATER_QUANTITY</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -15466,67 +15455,49 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>CUSTOM</t>
+        </is>
+      </c>
+      <c r="AB78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S78" t="n">
-        <v>0</v>
-      </c>
-      <c r="T78" t="n">
-        <v>10000</v>
-      </c>
-      <c r="U78" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V78" t="n">
-        <v>30</v>
-      </c>
-      <c r="W78" t="n">
-        <v>120</v>
-      </c>
-      <c r="X78" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF78" t="inlineStr">
         <is>
           <t>no</t>
@@ -15534,12 +15505,12 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AUDIO_VOLUME</t>
         </is>
       </c>
       <c r="AI78" t="inlineStr">
@@ -15591,22 +15562,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>HA Sensor (weight)</t>
+          <t>HA Switch</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ha-sensor-weight</t>
+          <t>ha-switch-none</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -15661,7 +15632,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -15671,67 +15642,49 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>DEVICE_LEVEL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S79" t="n">
-        <v>0</v>
-      </c>
-      <c r="T79" t="n">
-        <v>1000</v>
-      </c>
-      <c r="U79" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V79" t="n">
-        <v>30</v>
-      </c>
-      <c r="W79" t="n">
-        <v>120</v>
-      </c>
-      <c r="X79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF79" t="inlineStr">
         <is>
           <t>no</t>
@@ -15739,7 +15692,7 @@
       </c>
       <c r="AG79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH79" t="inlineStr">
@@ -15796,22 +15749,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>wind_speed</t>
+          <t>outlet</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HA Sensor (wind_speed)</t>
+          <t>HA Switch (outlet)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ha-sensor-wind_speed</t>
+          <t>ha-switch-outlet</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -15861,12 +15814,12 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>WIND_SPEED</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -15876,67 +15829,49 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>OUTDOOR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>ON_OFF</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>BINARY</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="S80" t="n">
-        <v>0</v>
-      </c>
-      <c r="T80" t="n">
-        <v>60</v>
-      </c>
-      <c r="U80" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V80" t="n">
-        <v>30</v>
-      </c>
-      <c r="W80" t="n">
-        <v>120</v>
-      </c>
-      <c r="X80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AF80" t="inlineStr">
         <is>
           <t>no</t>
@@ -15944,7 +15879,7 @@
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>POWER_STATE</t>
         </is>
       </c>
       <c r="AH80" t="inlineStr">
@@ -16001,22 +15936,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>siren</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HA Siren</t>
+          <t>HA Switch (switch)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>ha-siren-none</t>
+          <t>ha-switch-switch</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -16101,7 +16036,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>ON_OFF</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -16136,7 +16071,7 @@
       </c>
       <c r="AH81" t="inlineStr">
         <is>
-          <t>AUDIO_VOLUME</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AI81" t="inlineStr">
@@ -16188,7 +16123,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -16198,12 +16133,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>HA Switch</t>
+          <t>HA Valve</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>ha-switch-none</t>
+          <t>ha-valve-none</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -16218,7 +16153,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -16308,7 +16243,7 @@
       </c>
       <c r="AE82" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF82" t="inlineStr">
@@ -16375,22 +16310,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>outlet</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HA Switch (outlet)</t>
+          <t>HA Valve (gas)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ha-switch-outlet</t>
+          <t>ha-valve-gas</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -16405,7 +16340,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -16495,7 +16430,7 @@
       </c>
       <c r="AE83" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF83" t="inlineStr">
@@ -16562,22 +16497,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>valve</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>water</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>HA Switch (switch)</t>
+          <t>HA Valve (water)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ha-switch-switch</t>
+          <t>ha-valve-water</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -16592,7 +16527,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -16662,7 +16597,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -16677,22 +16612,22 @@
       </c>
       <c r="AD84" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>GRADUAL</t>
         </is>
       </c>
       <c r="AE84" t="inlineStr">
         <is>
-          <t>JOKER</t>
+          <t>HEATING</t>
         </is>
       </c>
       <c r="AF84" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>WATER_FLOW_RATE</t>
         </is>
       </c>
       <c r="AH84" t="inlineStr">
@@ -16754,17 +16689,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>water_heater</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>HA Valve</t>
+          <t>HA Valve (water_heater)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ha-valve-none</t>
+          <t>ha-valve-water_heater</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -16849,7 +16784,7 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>ON_OFF</t>
+          <t>POSITIONAL</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr">
@@ -16864,7 +16799,7 @@
       </c>
       <c r="AD85" t="inlineStr">
         <is>
-          <t>BINARY</t>
+          <t>GRADUAL</t>
         </is>
       </c>
       <c r="AE85" t="inlineStr">
@@ -16874,12 +16809,12 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t>POWER_STATE</t>
+          <t>WATER_FLOW_RATE</t>
         </is>
       </c>
       <c r="AH85" t="inlineStr">
@@ -16928,567 +16863,6 @@
         </is>
       </c>
       <c r="AQ85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>gas</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>HA Valve (gas)</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>ha-valve-gas</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA86" t="inlineStr">
-        <is>
-          <t>ON_OFF</t>
-        </is>
-      </c>
-      <c r="AB86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC86" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD86" t="inlineStr">
-        <is>
-          <t>BINARY</t>
-        </is>
-      </c>
-      <c r="AE86" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AG86" t="inlineStr">
-        <is>
-          <t>POWER_STATE</t>
-        </is>
-      </c>
-      <c r="AH86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN86" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>water</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>HA Valve (water)</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>ha-valve-water</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA87" t="inlineStr">
-        <is>
-          <t>POSITIONAL</t>
-        </is>
-      </c>
-      <c r="AB87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC87" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD87" t="inlineStr">
-        <is>
-          <t>GRADUAL</t>
-        </is>
-      </c>
-      <c r="AE87" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF87" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG87" t="inlineStr">
-        <is>
-          <t>WATER_FLOW_RATE</t>
-        </is>
-      </c>
-      <c r="AH87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN87" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ87" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>valve</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>water_heater</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>HA Valve (water_heater)</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>ha-valve-water_heater</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Home Assistant</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Q88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AA88" t="inlineStr">
-        <is>
-          <t>POSITIONAL</t>
-        </is>
-      </c>
-      <c r="AB88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AC88" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD88" t="inlineStr">
-        <is>
-          <t>GRADUAL</t>
-        </is>
-      </c>
-      <c r="AE88" t="inlineStr">
-        <is>
-          <t>HEATING</t>
-        </is>
-      </c>
-      <c r="AF88" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AG88" t="inlineStr">
-        <is>
-          <t>WATER_FLOW_RATE</t>
-        </is>
-      </c>
-      <c r="AH88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AI88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN88" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP88" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ88" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Plan and mapping excel Update
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ85"/>
+  <dimension ref="A1:AR85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -702,6 +702,11 @@
           <t>button.mode.VALUE</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>sensor.ds_unit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9631,6 +9636,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR49" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9836,6 +9846,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR50" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -10041,6 +10056,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10246,6 +10266,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>hPa</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10451,6 +10476,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -10656,6 +10686,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>ppm</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10861,6 +10896,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR55" t="inlineStr">
+        <is>
+          <t>ppm</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11066,6 +11106,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11271,6 +11316,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR57" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11476,6 +11526,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR58" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -11681,6 +11736,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR59" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -11886,6 +11946,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR60" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12091,6 +12156,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12296,6 +12366,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR62" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12501,6 +12576,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t>lx</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12706,6 +12786,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12911,6 +12996,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t>µg/m³</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -13116,6 +13206,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t>µg/m³</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -13321,6 +13416,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t>µg/m³</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -13526,6 +13626,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -13731,6 +13836,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR69" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -13936,6 +14046,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -14141,6 +14256,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>dB</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -14346,6 +14466,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -14551,6 +14676,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14756,6 +14886,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR74" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -14961,6 +15096,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -15166,6 +15306,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR76" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -15369,6 +15514,11 @@
       <c r="AQ77" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="AR77" t="inlineStr">
+        <is>
+          <t>m/s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix outputUsage = 0 for all types of grey output devices
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR85"/>
+  <dimension ref="A1:AX85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -677,32 +677,62 @@
           <t>output.ch5.channel_type.VALUE</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>output.ch0.resolution</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>output.ch1.resolution</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>output.ch2.resolution</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>output.ch3.resolution</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>output.ch4.resolution</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>output.ch5.resolution</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>button.button_type.VALUE</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>button.group.USER</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>button.group.VALUE</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>button.function.VALUE</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>button.mode.VALUE</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>sensor.ds_unit</t>
         </is>
@@ -869,27 +899,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1056,27 +1086,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1243,27 +1273,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1430,27 +1460,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1617,27 +1647,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ6" t="inlineStr">
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1804,27 +1834,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr">
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1991,27 +2021,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN8" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2178,27 +2208,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2365,27 +2395,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ10" t="inlineStr">
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2552,27 +2582,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ11" t="inlineStr">
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2739,27 +2769,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN12" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr">
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2926,27 +2956,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3113,27 +3143,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ14" t="inlineStr">
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3300,27 +3330,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ15" t="inlineStr">
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3487,27 +3517,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN16" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ16" t="inlineStr">
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3674,27 +3704,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN17" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ17" t="inlineStr">
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3861,27 +3891,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN18" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ18" t="inlineStr">
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4048,27 +4078,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ19" t="inlineStr">
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4235,27 +4265,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN20" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ20" t="inlineStr">
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4422,27 +4452,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ21" t="inlineStr">
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4609,27 +4639,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN22" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ22" t="inlineStr">
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4796,27 +4826,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ23" t="inlineStr">
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4983,27 +5013,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN24" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ24" t="inlineStr">
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5170,27 +5200,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN25" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ25" t="inlineStr">
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5357,27 +5387,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN26" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ26" t="inlineStr">
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW26" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5544,27 +5574,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ27" t="inlineStr">
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5731,27 +5761,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN28" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ28" t="inlineStr">
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5918,27 +5948,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN29" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ29" t="inlineStr">
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW29" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6105,27 +6135,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN30" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ30" t="inlineStr">
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6292,27 +6322,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM31" t="inlineStr">
+      <c r="AS31" t="inlineStr">
         <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="AN31" t="inlineStr">
+      <c r="AT31" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AO31" t="inlineStr">
+      <c r="AU31" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="AP31" t="inlineStr">
+      <c r="AV31" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AQ31" t="inlineStr">
+      <c r="AW31" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -6429,10 +6459,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC32" t="inlineStr">
-        <is>
-          <t>OUTDOORS</t>
-        </is>
+      <c r="AC32" t="n">
+        <v>0</v>
       </c>
       <c r="AD32" t="inlineStr">
         <is>
@@ -6481,25 +6509,30 @@
       </c>
       <c r="AM32" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN32" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ32" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW32" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6613,29 +6646,27 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>GRADUAL</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>BLINDS</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AC33" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
-      </c>
-      <c r="AD33" t="inlineStr">
-        <is>
-          <t>GRADUAL</t>
-        </is>
-      </c>
-      <c r="AE33" t="inlineStr">
-        <is>
-          <t>BLINDS</t>
-        </is>
-      </c>
-      <c r="AF33" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="AG33" t="inlineStr">
         <is>
           <t>SHADE_POSITION_INDOOR</t>
@@ -6668,25 +6699,35 @@
       </c>
       <c r="AM33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100/65536</t>
         </is>
       </c>
       <c r="AN33" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ33" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW33" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6803,10 +6844,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC34" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
+      <c r="AC34" t="n">
+        <v>0</v>
       </c>
       <c r="AD34" t="inlineStr">
         <is>
@@ -6855,25 +6894,30 @@
       </c>
       <c r="AM34" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN34" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ34" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW34" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6990,10 +7034,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC35" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
+      <c r="AC35" t="n">
+        <v>0</v>
       </c>
       <c r="AD35" t="inlineStr">
         <is>
@@ -7042,25 +7084,30 @@
       </c>
       <c r="AM35" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN35" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ35" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7177,10 +7224,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC36" t="inlineStr">
-        <is>
-          <t>OUTDOORS</t>
-        </is>
+      <c r="AC36" t="n">
+        <v>0</v>
       </c>
       <c r="AD36" t="inlineStr">
         <is>
@@ -7232,22 +7277,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AN36" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ36" t="inlineStr">
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW36" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7364,10 +7414,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC37" t="inlineStr">
-        <is>
-          <t>OUTDOORS</t>
-        </is>
+      <c r="AC37" t="n">
+        <v>0</v>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
@@ -7419,22 +7467,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AN37" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ37" t="inlineStr">
+      <c r="AS37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW37" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7551,10 +7604,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC38" t="inlineStr">
-        <is>
-          <t>OUTDOORS</t>
-        </is>
+      <c r="AC38" t="n">
+        <v>0</v>
       </c>
       <c r="AD38" t="inlineStr">
         <is>
@@ -7603,25 +7654,30 @@
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN38" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ38" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7738,10 +7794,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC39" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
+      <c r="AC39" t="n">
+        <v>0</v>
       </c>
       <c r="AD39" t="inlineStr">
         <is>
@@ -7790,25 +7844,30 @@
       </c>
       <c r="AM39" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN39" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ39" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7925,10 +7984,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC40" t="inlineStr">
-        <is>
-          <t>OUTDOORS</t>
-        </is>
+      <c r="AC40" t="n">
+        <v>0</v>
       </c>
       <c r="AD40" t="inlineStr">
         <is>
@@ -7977,25 +8034,35 @@
       </c>
       <c r="AM40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100/65536</t>
         </is>
       </c>
       <c r="AN40" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ40" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW40" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8112,10 +8179,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC41" t="inlineStr">
-        <is>
-          <t>ROOM</t>
-        </is>
+      <c r="AC41" t="n">
+        <v>0</v>
       </c>
       <c r="AD41" t="inlineStr">
         <is>
@@ -8164,25 +8229,30 @@
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN41" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ41" t="inlineStr">
+          <t>100/65536</t>
+        </is>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW41" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8349,27 +8419,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM42" t="inlineStr">
+      <c r="AS42" t="inlineStr">
         <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="AN42" t="inlineStr">
+      <c r="AT42" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="AO42" t="inlineStr">
+      <c r="AU42" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="AP42" t="inlineStr">
+      <c r="AV42" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AQ42" t="inlineStr">
+      <c r="AW42" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -8536,27 +8606,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM43" t="inlineStr">
+      <c r="AS43" t="inlineStr">
         <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="AN43" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO43" t="inlineStr">
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU43" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="AP43" t="inlineStr">
+      <c r="AV43" t="inlineStr">
         <is>
           <t>DOOR_BELL</t>
         </is>
       </c>
-      <c r="AQ43" t="inlineStr">
+      <c r="AW43" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -8723,27 +8793,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN44" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ44" t="inlineStr">
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW44" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8910,27 +8980,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN45" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ45" t="inlineStr">
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW45" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9032,27 +9102,27 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AM46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN46" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ46" t="inlineStr">
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW46" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9219,27 +9289,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN47" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ47" t="inlineStr">
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW47" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9406,27 +9476,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN48" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ48" t="inlineStr">
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW48" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9611,32 +9681,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR49" t="inlineStr">
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX49" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
@@ -9821,32 +9891,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR50" t="inlineStr">
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX50" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
@@ -10031,32 +10101,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN51" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR51" t="inlineStr">
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX51" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10241,32 +10311,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN52" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR52" t="inlineStr">
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX52" t="inlineStr">
         <is>
           <t>hPa</t>
         </is>
@@ -10451,32 +10521,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN53" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR53" t="inlineStr">
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX53" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -10661,32 +10731,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN54" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR54" t="inlineStr">
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX54" t="inlineStr">
         <is>
           <t>ppm</t>
         </is>
@@ -10871,32 +10941,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN55" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR55" t="inlineStr">
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT55" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX55" t="inlineStr">
         <is>
           <t>ppm</t>
         </is>
@@ -11081,32 +11151,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN56" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR56" t="inlineStr">
+      <c r="AS56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX56" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -11291,32 +11361,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN57" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR57" t="inlineStr">
+      <c r="AS57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX57" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
@@ -11501,32 +11571,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN58" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR58" t="inlineStr">
+      <c r="AS58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX58" t="inlineStr">
         <is>
           <t>s</t>
         </is>
@@ -11711,32 +11781,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN59" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR59" t="inlineStr">
+      <c r="AS59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX59" t="inlineStr">
         <is>
           <t>kWh</t>
         </is>
@@ -11921,32 +11991,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN60" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR60" t="inlineStr">
+      <c r="AS60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT60" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX60" t="inlineStr">
         <is>
           <t>Hz</t>
         </is>
@@ -12131,32 +12201,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN61" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR61" t="inlineStr">
+      <c r="AS61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX61" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12341,32 +12411,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN62" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR62" t="inlineStr">
+      <c r="AS62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX62" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -12551,32 +12621,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN63" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR63" t="inlineStr">
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX63" t="inlineStr">
         <is>
           <t>lx</t>
         </is>
@@ -12761,32 +12831,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN64" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR64" t="inlineStr">
+      <c r="AS64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX64" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12971,32 +13041,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN65" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR65" t="inlineStr">
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX65" t="inlineStr">
         <is>
           <t>µg/m³</t>
         </is>
@@ -13181,32 +13251,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN66" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR66" t="inlineStr">
+      <c r="AS66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX66" t="inlineStr">
         <is>
           <t>µg/m³</t>
         </is>
@@ -13391,32 +13461,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN67" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR67" t="inlineStr">
+      <c r="AS67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX67" t="inlineStr">
         <is>
           <t>µg/m³</t>
         </is>
@@ -13601,32 +13671,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN68" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR68" t="inlineStr">
+      <c r="AS68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX68" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -13811,32 +13881,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN69" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR69" t="inlineStr">
+      <c r="AS69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX69" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -14021,32 +14091,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN70" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR70" t="inlineStr">
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX70" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
@@ -14231,32 +14301,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN71" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR71" t="inlineStr">
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX71" t="inlineStr">
         <is>
           <t>dB</t>
         </is>
@@ -14441,32 +14511,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN72" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR72" t="inlineStr">
+      <c r="AS72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX72" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14651,32 +14721,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN73" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR73" t="inlineStr">
+      <c r="AS73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX73" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
@@ -14861,32 +14931,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN74" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR74" t="inlineStr">
+      <c r="AS74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX74" t="inlineStr">
         <is>
           <t>V</t>
         </is>
@@ -15071,32 +15141,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN75" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR75" t="inlineStr">
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX75" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -15281,32 +15351,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN76" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR76" t="inlineStr">
+      <c r="AS76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX76" t="inlineStr">
         <is>
           <t>g</t>
         </is>
@@ -15491,32 +15561,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN77" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AR77" t="inlineStr">
+      <c r="AS77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AX77" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -15683,27 +15753,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN78" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ78" t="inlineStr">
+      <c r="AS78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW78" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15870,27 +15940,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN79" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ79" t="inlineStr">
+      <c r="AS79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW79" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16057,27 +16127,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN80" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ80" t="inlineStr">
+      <c r="AS80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW80" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16244,27 +16314,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN81" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ81" t="inlineStr">
+      <c r="AS81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW81" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16431,27 +16501,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN82" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ82" t="inlineStr">
+      <c r="AS82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW82" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16618,27 +16688,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN83" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ83" t="inlineStr">
+      <c r="AS83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW83" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16805,27 +16875,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN84" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ84" t="inlineStr">
+      <c r="AS84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW84" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16992,27 +17062,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AM85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN85" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AO85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AQ85" t="inlineStr">
+      <c r="AS85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AT85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AU85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AV85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AW85" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
chore: regenerate mapping Excel with pydsvdcapi 0.8.9 new columns
</commit_message>
<xml_diff>
--- a/documents/ha_vdsd_mapping.xlsx
+++ b/documents/ha_vdsd_mapping.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE85"/>
+  <dimension ref="A1:BN85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -493,11 +493,20 @@
     <col width="22" customWidth="1" min="50" max="50"/>
     <col width="23" customWidth="1" min="51" max="51"/>
     <col width="22" customWidth="1" min="52" max="52"/>
-    <col width="26" customWidth="1" min="53" max="53"/>
-    <col width="19" customWidth="1" min="54" max="54"/>
-    <col width="20" customWidth="1" min="55" max="55"/>
-    <col width="23" customWidth="1" min="56" max="56"/>
-    <col width="19" customWidth="1" min="57" max="57"/>
+    <col width="28" customWidth="1" min="53" max="53"/>
+    <col width="40" customWidth="1" min="54" max="54"/>
+    <col width="34" customWidth="1" min="55" max="55"/>
+    <col width="18" customWidth="1" min="56" max="56"/>
+    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="58" max="58"/>
+    <col width="24" customWidth="1" min="59" max="59"/>
+    <col width="22" customWidth="1" min="60" max="60"/>
+    <col width="24" customWidth="1" min="61" max="61"/>
+    <col width="26" customWidth="1" min="62" max="62"/>
+    <col width="19" customWidth="1" min="63" max="63"/>
+    <col width="20" customWidth="1" min="64" max="64"/>
+    <col width="23" customWidth="1" min="65" max="65"/>
+    <col width="19" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -761,27 +770,72 @@
           <t>output.stopDelayTime</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>output.active_cooling_mode</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>output.heating_system_capability.VALUE</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>output.heating_system_type.VALUE</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeUp</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeDown</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeUpAlt1</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeDownAlt1</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeUpAlt2</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>output.dimTimeDownAlt2</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>button.button_type.VALUE</t>
         </is>
       </c>
-      <c r="BB1" s="2" t="inlineStr">
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>button.group.USER</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>button.group.VALUE</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>button.function.VALUE</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>button.mode.VALUE</t>
         </is>
@@ -995,12 +1049,12 @@
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC2" t="inlineStr">
@@ -1008,12 +1062,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1227,12 +1296,12 @@
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC3" t="inlineStr">
@@ -1240,12 +1309,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE3" t="inlineStr">
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1459,12 +1543,12 @@
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC4" t="inlineStr">
@@ -1472,12 +1556,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE4" t="inlineStr">
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1691,12 +1790,12 @@
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC5" t="inlineStr">
@@ -1704,12 +1803,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE5" t="inlineStr">
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1923,12 +2037,12 @@
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC6" t="inlineStr">
@@ -1936,12 +2050,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE6" t="inlineStr">
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2155,12 +2284,12 @@
       </c>
       <c r="BA7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC7" t="inlineStr">
@@ -2168,12 +2297,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE7" t="inlineStr">
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2387,12 +2531,12 @@
       </c>
       <c r="BA8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC8" t="inlineStr">
@@ -2400,12 +2544,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE8" t="inlineStr">
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2619,12 +2778,12 @@
       </c>
       <c r="BA9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC9" t="inlineStr">
@@ -2632,12 +2791,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE9" t="inlineStr">
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2851,12 +3025,12 @@
       </c>
       <c r="BA10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC10" t="inlineStr">
@@ -2864,12 +3038,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE10" t="inlineStr">
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3083,12 +3272,12 @@
       </c>
       <c r="BA11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC11" t="inlineStr">
@@ -3096,12 +3285,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE11" t="inlineStr">
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3315,12 +3519,12 @@
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB12" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC12" t="inlineStr">
@@ -3328,12 +3532,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE12" t="inlineStr">
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3547,12 +3766,12 @@
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC13" t="inlineStr">
@@ -3560,12 +3779,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE13" t="inlineStr">
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3779,12 +4013,12 @@
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC14" t="inlineStr">
@@ -3792,12 +4026,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE14" t="inlineStr">
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4011,12 +4260,12 @@
       </c>
       <c r="BA15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC15" t="inlineStr">
@@ -4024,12 +4273,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE15" t="inlineStr">
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4243,12 +4507,12 @@
       </c>
       <c r="BA16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC16" t="inlineStr">
@@ -4256,12 +4520,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE16" t="inlineStr">
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4475,12 +4754,12 @@
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC17" t="inlineStr">
@@ -4488,12 +4767,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE17" t="inlineStr">
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4707,12 +5001,12 @@
       </c>
       <c r="BA18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC18" t="inlineStr">
@@ -4720,12 +5014,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE18" t="inlineStr">
+      <c r="BJ18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4939,12 +5248,12 @@
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB19" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC19" t="inlineStr">
@@ -4952,12 +5261,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE19" t="inlineStr">
+      <c r="BJ19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5171,12 +5495,12 @@
       </c>
       <c r="BA20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC20" t="inlineStr">
@@ -5184,12 +5508,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE20" t="inlineStr">
+      <c r="BJ20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5403,12 +5742,12 @@
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB21" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC21" t="inlineStr">
@@ -5416,12 +5755,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE21" t="inlineStr">
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5635,12 +5989,12 @@
       </c>
       <c r="BA22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB22" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC22" t="inlineStr">
@@ -5648,12 +6002,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE22" t="inlineStr">
+      <c r="BJ22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5867,12 +6236,12 @@
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC23" t="inlineStr">
@@ -5880,12 +6249,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE23" t="inlineStr">
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6099,12 +6483,12 @@
       </c>
       <c r="BA24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC24" t="inlineStr">
@@ -6112,12 +6496,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE24" t="inlineStr">
+      <c r="BJ24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN24" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6331,12 +6730,12 @@
       </c>
       <c r="BA25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB25" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC25" t="inlineStr">
@@ -6344,12 +6743,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE25" t="inlineStr">
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6563,12 +6977,12 @@
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB26" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC26" t="inlineStr">
@@ -6576,12 +6990,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE26" t="inlineStr">
+      <c r="BJ26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN26" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6795,12 +7224,12 @@
       </c>
       <c r="BA27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB27" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC27" t="inlineStr">
@@ -6808,12 +7237,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE27" t="inlineStr">
+      <c r="BJ27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7027,12 +7471,12 @@
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB28" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC28" t="inlineStr">
@@ -7040,12 +7484,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE28" t="inlineStr">
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7259,12 +7718,12 @@
       </c>
       <c r="BA29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB29" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC29" t="inlineStr">
@@ -7272,12 +7731,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE29" t="inlineStr">
+      <c r="BJ29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN29" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7491,12 +7965,12 @@
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB30" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC30" t="inlineStr">
@@ -7504,12 +7978,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE30" t="inlineStr">
+      <c r="BJ30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7723,25 +8212,40 @@
       </c>
       <c r="BA31" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BC31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BJ31" t="inlineStr">
+        <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="BB31" t="inlineStr">
+      <c r="BK31" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="BC31" t="inlineStr">
+      <c r="BL31" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="BD31" t="inlineStr">
+      <c r="BM31" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="BE31" t="inlineStr">
+      <c r="BN31" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -7955,12 +8459,12 @@
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC32" t="inlineStr">
@@ -7968,12 +8472,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE32" t="inlineStr">
+      <c r="BJ32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN32" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8187,12 +8706,12 @@
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB33" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC33" t="inlineStr">
@@ -8200,12 +8719,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE33" t="inlineStr">
+      <c r="BJ33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN33" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8419,12 +8953,12 @@
       </c>
       <c r="BA34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB34" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC34" t="inlineStr">
@@ -8432,12 +8966,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE34" t="inlineStr">
+      <c r="BJ34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN34" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8651,12 +9200,12 @@
       </c>
       <c r="BA35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB35" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC35" t="inlineStr">
@@ -8664,12 +9213,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE35" t="inlineStr">
+      <c r="BJ35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8883,12 +9447,12 @@
       </c>
       <c r="BA36" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB36" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC36" t="inlineStr">
@@ -8896,12 +9460,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE36" t="inlineStr">
+      <c r="BJ36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN36" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9115,12 +9694,12 @@
       </c>
       <c r="BA37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB37" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC37" t="inlineStr">
@@ -9128,12 +9707,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE37" t="inlineStr">
+      <c r="BJ37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK37" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN37" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9347,12 +9941,12 @@
       </c>
       <c r="BA38" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB38" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC38" t="inlineStr">
@@ -9360,12 +9954,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE38" t="inlineStr">
+      <c r="BJ38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK38" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN38" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9579,12 +10188,12 @@
       </c>
       <c r="BA39" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB39" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC39" t="inlineStr">
@@ -9592,12 +10201,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE39" t="inlineStr">
+      <c r="BJ39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9811,12 +10435,12 @@
       </c>
       <c r="BA40" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB40" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC40" t="inlineStr">
@@ -9824,12 +10448,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE40" t="inlineStr">
+      <c r="BJ40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK40" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN40" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10043,12 +10682,12 @@
       </c>
       <c r="BA41" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB41" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC41" t="inlineStr">
@@ -10056,12 +10695,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE41" t="inlineStr">
+      <c r="BJ41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK41" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN41" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10275,25 +10929,40 @@
       </c>
       <c r="BA42" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BC42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BJ42" t="inlineStr">
+        <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="BB42" t="inlineStr">
+      <c r="BK42" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="BC42" t="inlineStr">
+      <c r="BL42" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="BD42" t="inlineStr">
+      <c r="BM42" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="BE42" t="inlineStr">
+      <c r="BN42" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -10507,25 +11176,40 @@
       </c>
       <c r="BA43" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BB43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BC43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BJ43" t="inlineStr">
+        <is>
           <t>SINGLE_PUSHBUTTON</t>
         </is>
       </c>
-      <c r="BB43" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="BC43" t="inlineStr">
+      <c r="BK43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL43" t="inlineStr">
         <is>
           <t>JOKER</t>
         </is>
       </c>
-      <c r="BD43" t="inlineStr">
+      <c r="BM43" t="inlineStr">
         <is>
           <t>DOOR_BELL</t>
         </is>
       </c>
-      <c r="BE43" t="inlineStr">
+      <c r="BN43" t="inlineStr">
         <is>
           <t>STANDARD</t>
         </is>
@@ -10739,12 +11423,12 @@
       </c>
       <c r="BA44" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB44" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC44" t="inlineStr">
@@ -10752,12 +11436,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE44" t="inlineStr">
+      <c r="BJ44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN44" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10971,12 +11670,12 @@
       </c>
       <c r="BA45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB45" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC45" t="inlineStr">
@@ -10984,12 +11683,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE45" t="inlineStr">
+      <c r="BJ45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK45" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN45" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11203,12 +11917,12 @@
       </c>
       <c r="BA46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB46" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC46" t="inlineStr">
@@ -11216,12 +11930,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE46" t="inlineStr">
+      <c r="BJ46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN46" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11435,12 +12164,12 @@
       </c>
       <c r="BA47" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB47" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC47" t="inlineStr">
@@ -11448,12 +12177,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE47" t="inlineStr">
+      <c r="BJ47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK47" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN47" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11667,12 +12411,12 @@
       </c>
       <c r="BA48" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB48" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC48" t="inlineStr">
@@ -11680,12 +12424,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE48" t="inlineStr">
+      <c r="BJ48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN48" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11917,12 +12676,12 @@
       </c>
       <c r="BA49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB49" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC49" t="inlineStr">
@@ -11930,12 +12689,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE49" t="inlineStr">
+      <c r="BJ49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN49" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12167,12 +12941,12 @@
       </c>
       <c r="BA50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB50" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC50" t="inlineStr">
@@ -12180,12 +12954,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD50" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE50" t="inlineStr">
+      <c r="BJ50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN50" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12417,12 +13206,12 @@
       </c>
       <c r="BA51" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB51" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC51" t="inlineStr">
@@ -12430,12 +13219,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE51" t="inlineStr">
+      <c r="BJ51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN51" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12667,12 +13471,12 @@
       </c>
       <c r="BA52" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB52" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC52" t="inlineStr">
@@ -12680,12 +13484,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE52" t="inlineStr">
+      <c r="BJ52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN52" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12917,12 +13736,12 @@
       </c>
       <c r="BA53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB53" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC53" t="inlineStr">
@@ -12930,12 +13749,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD53" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE53" t="inlineStr">
+      <c r="BJ53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN53" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13167,12 +14001,12 @@
       </c>
       <c r="BA54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB54" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC54" t="inlineStr">
@@ -13180,12 +14014,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE54" t="inlineStr">
+      <c r="BJ54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN54" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13417,12 +14266,12 @@
       </c>
       <c r="BA55" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB55" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC55" t="inlineStr">
@@ -13430,12 +14279,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD55" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE55" t="inlineStr">
+      <c r="BJ55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK55" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN55" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13667,12 +14531,12 @@
       </c>
       <c r="BA56" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB56" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC56" t="inlineStr">
@@ -13680,12 +14544,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE56" t="inlineStr">
+      <c r="BJ56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN56" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13917,12 +14796,12 @@
       </c>
       <c r="BA57" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB57" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC57" t="inlineStr">
@@ -13930,12 +14809,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE57" t="inlineStr">
+      <c r="BJ57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN57" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14167,12 +15061,12 @@
       </c>
       <c r="BA58" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB58" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC58" t="inlineStr">
@@ -14180,12 +15074,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE58" t="inlineStr">
+      <c r="BJ58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN58" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14417,12 +15326,12 @@
       </c>
       <c r="BA59" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB59" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC59" t="inlineStr">
@@ -14430,12 +15339,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE59" t="inlineStr">
+      <c r="BJ59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK59" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN59" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14667,12 +15591,12 @@
       </c>
       <c r="BA60" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB60" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC60" t="inlineStr">
@@ -14680,12 +15604,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE60" t="inlineStr">
+      <c r="BJ60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK60" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN60" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14917,12 +15856,12 @@
       </c>
       <c r="BA61" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB61" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC61" t="inlineStr">
@@ -14930,12 +15869,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE61" t="inlineStr">
+      <c r="BJ61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN61" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15167,12 +16121,12 @@
       </c>
       <c r="BA62" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB62" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC62" t="inlineStr">
@@ -15180,12 +16134,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE62" t="inlineStr">
+      <c r="BJ62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN62" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15417,12 +16386,12 @@
       </c>
       <c r="BA63" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC63" t="inlineStr">
@@ -15430,12 +16399,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE63" t="inlineStr">
+      <c r="BJ63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN63" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15667,12 +16651,12 @@
       </c>
       <c r="BA64" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB64" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC64" t="inlineStr">
@@ -15680,12 +16664,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE64" t="inlineStr">
+      <c r="BJ64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN64" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15917,12 +16916,12 @@
       </c>
       <c r="BA65" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB65" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC65" t="inlineStr">
@@ -15930,12 +16929,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE65" t="inlineStr">
+      <c r="BJ65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN65" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16167,12 +17181,12 @@
       </c>
       <c r="BA66" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB66" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC66" t="inlineStr">
@@ -16180,12 +17194,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE66" t="inlineStr">
+      <c r="BJ66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN66" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16417,12 +17446,12 @@
       </c>
       <c r="BA67" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB67" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC67" t="inlineStr">
@@ -16430,12 +17459,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE67" t="inlineStr">
+      <c r="BJ67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN67" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16667,12 +17711,12 @@
       </c>
       <c r="BA68" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB68" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC68" t="inlineStr">
@@ -16680,12 +17724,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE68" t="inlineStr">
+      <c r="BJ68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN68" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16917,12 +17976,12 @@
       </c>
       <c r="BA69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB69" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC69" t="inlineStr">
@@ -16930,12 +17989,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE69" t="inlineStr">
+      <c r="BJ69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK69" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN69" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17167,12 +18241,12 @@
       </c>
       <c r="BA70" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB70" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC70" t="inlineStr">
@@ -17180,12 +18254,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE70" t="inlineStr">
+      <c r="BJ70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN70" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17417,12 +18506,12 @@
       </c>
       <c r="BA71" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB71" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC71" t="inlineStr">
@@ -17430,12 +18519,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE71" t="inlineStr">
+      <c r="BJ71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17667,12 +18771,12 @@
       </c>
       <c r="BA72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB72" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC72" t="inlineStr">
@@ -17680,12 +18784,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE72" t="inlineStr">
+      <c r="BJ72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN72" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17917,12 +19036,12 @@
       </c>
       <c r="BA73" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB73" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC73" t="inlineStr">
@@ -17930,12 +19049,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE73" t="inlineStr">
+      <c r="BJ73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN73" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18167,12 +19301,12 @@
       </c>
       <c r="BA74" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB74" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC74" t="inlineStr">
@@ -18180,12 +19314,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE74" t="inlineStr">
+      <c r="BJ74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18417,12 +19566,12 @@
       </c>
       <c r="BA75" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB75" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC75" t="inlineStr">
@@ -18430,12 +19579,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE75" t="inlineStr">
+      <c r="BJ75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN75" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18667,12 +19831,12 @@
       </c>
       <c r="BA76" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB76" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC76" t="inlineStr">
@@ -18680,12 +19844,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE76" t="inlineStr">
+      <c r="BJ76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN76" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18917,12 +20096,12 @@
       </c>
       <c r="BA77" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB77" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC77" t="inlineStr">
@@ -18930,12 +20109,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE77" t="inlineStr">
+      <c r="BJ77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN77" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19149,12 +20343,12 @@
       </c>
       <c r="BA78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB78" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC78" t="inlineStr">
@@ -19162,12 +20356,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE78" t="inlineStr">
+      <c r="BJ78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN78" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19381,12 +20590,12 @@
       </c>
       <c r="BA79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB79" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC79" t="inlineStr">
@@ -19394,12 +20603,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE79" t="inlineStr">
+      <c r="BJ79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN79" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19613,12 +20837,12 @@
       </c>
       <c r="BA80" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB80" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC80" t="inlineStr">
@@ -19626,12 +20850,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE80" t="inlineStr">
+      <c r="BJ80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN80" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19845,12 +21084,12 @@
       </c>
       <c r="BA81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB81" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC81" t="inlineStr">
@@ -19858,12 +21097,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE81" t="inlineStr">
+      <c r="BJ81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN81" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20077,12 +21331,12 @@
       </c>
       <c r="BA82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB82" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC82" t="inlineStr">
@@ -20090,12 +21344,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE82" t="inlineStr">
+      <c r="BJ82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN82" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20309,12 +21578,12 @@
       </c>
       <c r="BA83" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB83" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC83" t="inlineStr">
@@ -20322,12 +21591,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE83" t="inlineStr">
+      <c r="BJ83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN83" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20541,12 +21825,12 @@
       </c>
       <c r="BA84" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB84" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC84" t="inlineStr">
@@ -20554,12 +21838,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE84" t="inlineStr">
+      <c r="BJ84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN84" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20773,12 +22072,12 @@
       </c>
       <c r="BA85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>no</t>
         </is>
       </c>
       <c r="BB85" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="BC85" t="inlineStr">
@@ -20786,19 +22085,34 @@
           <t>-</t>
         </is>
       </c>
-      <c r="BD85" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="BE85" t="inlineStr">
+      <c r="BJ85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BK85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BL85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BM85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BN85" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="41">
+  <dataValidations count="44">
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$A$1:$A$2</formula1>
     </dataValidation>
@@ -20866,40 +22180,40 @@
       <formula1>_lookups!$A$1:$A$2</formula1>
     </dataValidation>
     <dataValidation sqref="AH2:AH1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AI2:AI1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AJ2:AJ1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AK2:AK1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AL2:AL1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AM2:AM1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AN2:AN1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AO2:AO1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AP2:AP1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AQ2:AQ1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AR2:AR1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AS2:AS1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>_lookups!$M$1:$M$28</formula1>
+      <formula1>_lookups!$M$1:$M$29</formula1>
     </dataValidation>
     <dataValidation sqref="AT2:AT1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$A$1:$A$2</formula1>
@@ -20908,18 +22222,27 @@
       <formula1>_lookups!$A$1:$A$2</formula1>
     </dataValidation>
     <dataValidation sqref="BA2:BA1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_lookups!$A$1:$A$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="BB2:BB1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_lookups!$R$1:$R$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="BC2:BC1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_lookups!$S$1:$S$8</formula1>
+    </dataValidation>
+    <dataValidation sqref="BJ2:BJ1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$N$1:$N$8</formula1>
     </dataValidation>
-    <dataValidation sqref="BB2:BB1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="BK2:BK1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$A$1:$A$2</formula1>
     </dataValidation>
-    <dataValidation sqref="BC2:BC1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="BL2:BL1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$O$1:$O$14</formula1>
     </dataValidation>
-    <dataValidation sqref="BD2:BD1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="BM2:BM1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$P$1:$P$6</formula1>
     </dataValidation>
-    <dataValidation sqref="BE2:BE1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="BN2:BN1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lookups!$Q$1:$Q$24</formula1>
     </dataValidation>
   </dataValidations>
@@ -20933,7 +22256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21022,6 +22345,16 @@
           <t>-</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -21109,6 +22442,16 @@
           <t>STANDARD</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>HEATING_ONLY</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>UNDEFINED</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -21191,6 +22534,16 @@
           <t>TURBO</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>COOLING_ONLY</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>FLOOR_HEATING</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -21273,6 +22626,16 @@
           <t>SWITCHED</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>HEATING_AND_COOLING</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>RADIATOR</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -21355,6 +22718,11 @@
           <t>TWO_WAY_DOWN_PAIRED_1</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>WALL_HEATING</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -21422,6 +22790,11 @@
           <t>TWO_WAY_DOWN_PAIRED_2</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>CONVECTOR_PASSIVE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
@@ -21484,6 +22857,11 @@
           <t>TWO_WAY_DOWN_PAIRED_3</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>CONVECTOR_ACTIVE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -21546,6 +22924,11 @@
           <t>TWO_WAY_DOWN_PAIRED_4</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>FLOOR_HEATING_LOW_ENERGY</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -22071,6 +23454,11 @@
       <c r="F29" t="inlineStr">
         <is>
           <t>WATER_QUANTITY</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>FCU_OPERATION_MODE</t>
         </is>
       </c>
     </row>

</xml_diff>